<commit_message>
Swap unrealistic call-center columns for survey-native categorical fields
handle_time_seconds / is_first_contact_resolution / is_repeat_contact_30d
live in a separate telephony/CRM system and would need a real operational
join - not something a CSAT survey table itself would realistically carry.
Replaced with plan_tier, circle, and survey_type: all genuine customer-
master / survey-platform attributes routinely pre-joined onto a survey
export by customer ID, no cross-system operational join implied.

Updated summary/chart sections, PPT deck content, narration numbers, and
CLAUDE.md's decision log to match. Regenerated and reverified end-to-end.
</commit_message>
<xml_diff>
--- a/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
+++ b/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="70">
   <si>
     <t>term</t>
   </si>
@@ -34,120 +34,120 @@
     <t>charged</t>
   </si>
   <si>
+    <t>issue</t>
+  </si>
+  <si>
+    <t>pack</t>
+  </si>
+  <si>
     <t>request</t>
   </si>
   <si>
-    <t>pack</t>
-  </si>
-  <si>
-    <t>issue</t>
-  </si>
-  <si>
     <t>explained</t>
   </si>
   <si>
+    <t>activation</t>
+  </si>
+  <si>
     <t>update</t>
   </si>
   <si>
+    <t>data</t>
+  </si>
+  <si>
     <t>data pack</t>
   </si>
   <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>activation</t>
+    <t>time</t>
+  </si>
+  <si>
+    <t>hi team</t>
   </si>
   <si>
     <t>team</t>
   </si>
   <si>
-    <t>hi team</t>
-  </si>
-  <si>
     <t>hi</t>
   </si>
   <si>
-    <t>time</t>
-  </si>
-  <si>
     <t>keeps</t>
   </si>
   <si>
+    <t>swap request</t>
+  </si>
+  <si>
+    <t>sim</t>
+  </si>
+  <si>
+    <t>sim swap</t>
+  </si>
+  <si>
+    <t>swap</t>
+  </si>
+  <si>
+    <t>pack activation</t>
+  </si>
+  <si>
+    <t>used</t>
+  </si>
+  <si>
+    <t>billing issue</t>
+  </si>
+  <si>
+    <t>billing</t>
+  </si>
+  <si>
+    <t>charged twice</t>
+  </si>
+  <si>
     <t>twice</t>
   </si>
   <si>
-    <t>charged twice</t>
+    <t>roaming</t>
+  </si>
+  <si>
+    <t>unexpected</t>
+  </si>
+  <si>
+    <t>agreed</t>
+  </si>
+  <si>
+    <t>invoice</t>
+  </si>
+  <si>
+    <t>shows</t>
+  </si>
+  <si>
+    <t>invoice shows</t>
   </si>
   <si>
     <t>fee</t>
   </si>
   <si>
-    <t>deducted</t>
+    <t>network</t>
+  </si>
+  <si>
+    <t>network issue</t>
+  </si>
+  <si>
+    <t>update request</t>
+  </si>
+  <si>
+    <t>address update</t>
+  </si>
+  <si>
+    <t>address</t>
   </si>
   <si>
     <t>deducted incorrectly</t>
   </si>
   <si>
-    <t>received</t>
-  </si>
-  <si>
-    <t>refund</t>
+    <t>incorrectly</t>
   </si>
   <si>
     <t>incorrectly received</t>
   </si>
   <si>
-    <t>received refund</t>
-  </si>
-  <si>
-    <t>incorrectly</t>
-  </si>
-  <si>
-    <t>shows</t>
-  </si>
-  <si>
-    <t>invoice shows</t>
-  </si>
-  <si>
-    <t>invoice</t>
-  </si>
-  <si>
-    <t>used</t>
-  </si>
-  <si>
-    <t>sim swap</t>
-  </si>
-  <si>
-    <t>swap</t>
-  </si>
-  <si>
-    <t>swap request</t>
-  </si>
-  <si>
-    <t>sim</t>
-  </si>
-  <si>
-    <t>roaming</t>
-  </si>
-  <si>
-    <t>address</t>
-  </si>
-  <si>
-    <t>address update</t>
-  </si>
-  <si>
-    <t>update request</t>
-  </si>
-  <si>
-    <t>unexpected</t>
-  </si>
-  <si>
-    <t>agreed</t>
-  </si>
-  <si>
-    <t>network</t>
-  </si>
-  <si>
     <t>agent helpful</t>
   </si>
   <si>
@@ -157,12 +157,6 @@
     <t>agent resolved</t>
   </si>
   <si>
-    <t>billing</t>
-  </si>
-  <si>
-    <t>billing issue</t>
-  </si>
-  <si>
     <t>clearly</t>
   </si>
   <si>
@@ -179,12 +173,6 @@
   </si>
   <si>
     <t>issue sorted</t>
-  </si>
-  <si>
-    <t>network issue</t>
-  </si>
-  <si>
-    <t>pack activation</t>
   </si>
   <si>
     <t>polite</t>
@@ -567,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -589,13 +577,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>1135</v>
+        <v>1117</v>
       </c>
       <c r="C2">
-        <v>1796</v>
+        <v>1879</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -603,13 +591,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>749</v>
+        <v>720</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -617,13 +605,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>711</v>
+        <v>705</v>
       </c>
       <c r="C4">
-        <v>626</v>
+        <v>1098</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -631,13 +619,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>678</v>
+        <v>702</v>
       </c>
       <c r="C5">
-        <v>783</v>
+        <v>762</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -645,13 +633,13 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>662</v>
+        <v>700</v>
       </c>
       <c r="C6">
-        <v>1142</v>
+        <v>646</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -659,13 +647,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>642</v>
+        <v>663</v>
       </c>
       <c r="C7">
-        <v>674</v>
+        <v>704</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -673,13 +661,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>561</v>
+        <v>546</v>
       </c>
       <c r="C8">
-        <v>388</v>
+        <v>368</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -687,13 +675,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>508</v>
+        <v>545</v>
       </c>
       <c r="C9">
-        <v>563</v>
+        <v>399</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -701,13 +689,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>508</v>
+        <v>531</v>
       </c>
       <c r="C10">
-        <v>563</v>
+        <v>521</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -715,13 +703,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>495</v>
+        <v>531</v>
       </c>
       <c r="C11">
-        <v>394</v>
+        <v>521</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -729,13 +717,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>483</v>
+        <v>514</v>
       </c>
       <c r="C12">
-        <v>656</v>
+        <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -743,13 +731,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>483</v>
+        <v>502</v>
       </c>
       <c r="C13">
-        <v>656</v>
+        <v>686</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -757,13 +745,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>483</v>
+        <v>502</v>
       </c>
       <c r="C14">
-        <v>656</v>
+        <v>686</v>
       </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -771,13 +759,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>477</v>
+        <v>502</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>686</v>
       </c>
       <c r="D15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -785,13 +773,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>414</v>
+        <v>473</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -799,13 +787,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -813,13 +801,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -830,10 +818,10 @@
         <v>372</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -841,13 +829,13 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -855,13 +843,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -869,13 +857,13 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -883,13 +871,13 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>325</v>
       </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -897,13 +885,13 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -911,13 +899,13 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -925,13 +913,13 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -939,13 +927,13 @@
         <v>29</v>
       </c>
       <c r="B27">
-        <v>368</v>
+        <v>351</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -953,13 +941,13 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -967,13 +955,13 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -981,13 +969,13 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>367</v>
+        <v>350</v>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -995,13 +983,13 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1009,13 +997,13 @@
         <v>34</v>
       </c>
       <c r="B32">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1023,13 +1011,13 @@
         <v>35</v>
       </c>
       <c r="B33">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1037,13 +1025,13 @@
         <v>36</v>
       </c>
       <c r="B34">
-        <v>361</v>
+        <v>347</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1051,13 +1039,13 @@
         <v>37</v>
       </c>
       <c r="B35">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="C35">
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1065,13 +1053,13 @@
         <v>38</v>
       </c>
       <c r="B36">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="C36">
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1079,13 +1067,13 @@
         <v>39</v>
       </c>
       <c r="B37">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="C37">
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1093,13 +1081,13 @@
         <v>40</v>
       </c>
       <c r="B38">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="C38">
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -1107,13 +1095,13 @@
         <v>41</v>
       </c>
       <c r="B39">
-        <v>346</v>
+        <v>325</v>
       </c>
       <c r="C39">
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -1121,13 +1109,13 @@
         <v>42</v>
       </c>
       <c r="B40">
-        <v>346</v>
+        <v>325</v>
       </c>
       <c r="C40">
         <v>0</v>
       </c>
       <c r="D40" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -1135,13 +1123,13 @@
         <v>43</v>
       </c>
       <c r="B41">
-        <v>343</v>
+        <v>325</v>
       </c>
       <c r="C41">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D41" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1152,10 +1140,10 @@
         <v>0</v>
       </c>
       <c r="C42">
-        <v>397</v>
+        <v>476</v>
       </c>
       <c r="D42" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -1166,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="C43">
-        <v>434</v>
+        <v>454</v>
       </c>
       <c r="D43" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1180,10 +1168,10 @@
         <v>0</v>
       </c>
       <c r="C44">
-        <v>518</v>
+        <v>497</v>
       </c>
       <c r="D44" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1194,10 +1182,10 @@
         <v>0</v>
       </c>
       <c r="C45">
-        <v>347</v>
+        <v>454</v>
       </c>
       <c r="D45" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1208,10 +1196,10 @@
         <v>0</v>
       </c>
       <c r="C46">
-        <v>347</v>
+        <v>457</v>
       </c>
       <c r="D46" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1222,10 +1210,10 @@
         <v>0</v>
       </c>
       <c r="C47">
-        <v>434</v>
+        <v>457</v>
       </c>
       <c r="D47" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1236,10 +1224,10 @@
         <v>0</v>
       </c>
       <c r="C48">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="D48" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -1250,10 +1238,10 @@
         <v>0</v>
       </c>
       <c r="C49">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="D49" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -1264,10 +1252,10 @@
         <v>0</v>
       </c>
       <c r="C50">
-        <v>397</v>
+        <v>457</v>
       </c>
       <c r="D50" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1278,10 +1266,10 @@
         <v>0</v>
       </c>
       <c r="C51">
-        <v>397</v>
+        <v>951</v>
       </c>
       <c r="D51" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -1292,10 +1280,10 @@
         <v>0</v>
       </c>
       <c r="C52">
-        <v>465</v>
+        <v>454</v>
       </c>
       <c r="D52" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -1306,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="C53">
-        <v>330</v>
+        <v>476</v>
       </c>
       <c r="D53" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -1320,10 +1308,10 @@
         <v>0</v>
       </c>
       <c r="C54">
-        <v>332</v>
+        <v>414</v>
       </c>
       <c r="D54" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -1334,10 +1322,10 @@
         <v>0</v>
       </c>
       <c r="C55">
-        <v>952</v>
+        <v>414</v>
       </c>
       <c r="D55" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -1348,10 +1336,10 @@
         <v>0</v>
       </c>
       <c r="C56">
-        <v>434</v>
+        <v>497</v>
       </c>
       <c r="D56" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -1362,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="C57">
-        <v>397</v>
+        <v>497</v>
       </c>
       <c r="D57" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -1376,10 +1364,10 @@
         <v>0</v>
       </c>
       <c r="C58">
-        <v>446</v>
+        <v>496</v>
       </c>
       <c r="D58" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -1390,10 +1378,10 @@
         <v>0</v>
       </c>
       <c r="C59">
-        <v>446</v>
+        <v>580</v>
       </c>
       <c r="D59" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -1404,10 +1392,10 @@
         <v>0</v>
       </c>
       <c r="C60">
-        <v>518</v>
+        <v>476</v>
       </c>
       <c r="D60" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -1418,10 +1406,10 @@
         <v>0</v>
       </c>
       <c r="C61">
-        <v>518</v>
+        <v>476</v>
       </c>
       <c r="D61" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -1432,10 +1420,10 @@
         <v>0</v>
       </c>
       <c r="C62">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="D62" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -1446,10 +1434,10 @@
         <v>0</v>
       </c>
       <c r="C63">
-        <v>607</v>
+        <v>457</v>
       </c>
       <c r="D63" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -1460,66 +1448,10 @@
         <v>0</v>
       </c>
       <c r="C64">
-        <v>397</v>
+        <v>414</v>
       </c>
       <c r="D64" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4">
-      <c r="A65" t="s">
-        <v>67</v>
-      </c>
-      <c r="B65">
-        <v>0</v>
-      </c>
-      <c r="C65">
-        <v>397</v>
-      </c>
-      <c r="D65" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4">
-      <c r="A66" t="s">
-        <v>68</v>
-      </c>
-      <c r="B66">
-        <v>0</v>
-      </c>
-      <c r="C66">
-        <v>526</v>
-      </c>
-      <c r="D66" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4">
-      <c r="A67" t="s">
-        <v>69</v>
-      </c>
-      <c r="B67">
-        <v>0</v>
-      </c>
-      <c r="C67">
-        <v>465</v>
-      </c>
-      <c r="D67" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4">
-      <c r="A68" t="s">
-        <v>70</v>
-      </c>
-      <c r="B68">
-        <v>0</v>
-      </c>
-      <c r="C68">
-        <v>446</v>
-      </c>
-      <c r="D68" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Drop survey_type, expand plan_tier to 5 options and circle to all 23 states
survey_type wasn't the right column per feedback - removed entirely.
plan_tier is now a flat 5-value list (Basic/Standard/Plus/Premium/Elite)
shared across LoBs instead of 2 LoB-tied options. circle now covers all
23 official Indian telecom circles (DoT-licensed service areas), which
collectively map to every state/UT, instead of an arbitrary 5-state list.

Updated summary/chart sections (15 charts now), PPT deck, narration
numbers, and CLAUDE.md's decision log to match. Regenerated end-to-end.
</commit_message>
<xml_diff>
--- a/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
+++ b/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="72">
   <si>
     <t>term</t>
   </si>
@@ -37,178 +37,184 @@
     <t>issue</t>
   </si>
   <si>
+    <t>request</t>
+  </si>
+  <si>
     <t>pack</t>
   </si>
   <si>
-    <t>request</t>
-  </si>
-  <si>
     <t>explained</t>
   </si>
   <si>
+    <t>team</t>
+  </si>
+  <si>
+    <t>hi team</t>
+  </si>
+  <si>
+    <t>hi</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>data pack</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
     <t>activation</t>
   </si>
   <si>
-    <t>update</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>data pack</t>
-  </si>
-  <si>
     <t>time</t>
   </si>
   <si>
-    <t>hi team</t>
-  </si>
-  <si>
-    <t>team</t>
-  </si>
-  <si>
-    <t>hi</t>
-  </si>
-  <si>
     <t>keeps</t>
   </si>
   <si>
+    <t>roaming</t>
+  </si>
+  <si>
+    <t>agreed</t>
+  </si>
+  <si>
+    <t>unexpected</t>
+  </si>
+  <si>
+    <t>charged twice</t>
+  </si>
+  <si>
+    <t>twice</t>
+  </si>
+  <si>
+    <t>used</t>
+  </si>
+  <si>
+    <t>billing</t>
+  </si>
+  <si>
+    <t>billing issue</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>shows</t>
+  </si>
+  <si>
+    <t>invoice shows</t>
+  </si>
+  <si>
+    <t>update request</t>
+  </si>
+  <si>
+    <t>invoice</t>
+  </si>
+  <si>
+    <t>address update</t>
+  </si>
+  <si>
+    <t>fee</t>
+  </si>
+  <si>
+    <t>received</t>
+  </si>
+  <si>
+    <t>deducted</t>
+  </si>
+  <si>
+    <t>deducted incorrectly</t>
+  </si>
+  <si>
+    <t>refund</t>
+  </si>
+  <si>
+    <t>incorrectly received</t>
+  </si>
+  <si>
+    <t>incorrectly</t>
+  </si>
+  <si>
+    <t>received refund</t>
+  </si>
+  <si>
     <t>swap request</t>
   </si>
   <si>
+    <t>swap</t>
+  </si>
+  <si>
+    <t>sim swap</t>
+  </si>
+  <si>
+    <t>agent helpful</t>
+  </si>
+  <si>
+    <t>agent polite</t>
+  </si>
+  <si>
+    <t>agent resolved</t>
+  </si>
+  <si>
+    <t>clearly</t>
+  </si>
+  <si>
+    <t>great</t>
+  </si>
+  <si>
+    <t>great service</t>
+  </si>
+  <si>
+    <t>helpful</t>
+  </si>
+  <si>
+    <t>helpful professional</t>
+  </si>
+  <si>
+    <t>issue sorted</t>
+  </si>
+  <si>
+    <t>network issue</t>
+  </si>
+  <si>
+    <t>polite</t>
+  </si>
+  <si>
+    <t>polite explained</t>
+  </si>
+  <si>
+    <t>professional</t>
+  </si>
+  <si>
+    <t>quick</t>
+  </si>
+  <si>
+    <t>quick resolution</t>
+  </si>
+  <si>
+    <t>quickly</t>
+  </si>
+  <si>
+    <t>quickly polite</t>
+  </si>
+  <si>
+    <t>resolution</t>
+  </si>
+  <si>
+    <t>resolved</t>
+  </si>
+  <si>
+    <t>satisfied</t>
+  </si>
+  <si>
+    <t>satisfied agent</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
     <t>sim</t>
-  </si>
-  <si>
-    <t>sim swap</t>
-  </si>
-  <si>
-    <t>swap</t>
-  </si>
-  <si>
-    <t>pack activation</t>
-  </si>
-  <si>
-    <t>used</t>
-  </si>
-  <si>
-    <t>billing issue</t>
-  </si>
-  <si>
-    <t>billing</t>
-  </si>
-  <si>
-    <t>charged twice</t>
-  </si>
-  <si>
-    <t>twice</t>
-  </si>
-  <si>
-    <t>roaming</t>
-  </si>
-  <si>
-    <t>unexpected</t>
-  </si>
-  <si>
-    <t>agreed</t>
-  </si>
-  <si>
-    <t>invoice</t>
-  </si>
-  <si>
-    <t>shows</t>
-  </si>
-  <si>
-    <t>invoice shows</t>
-  </si>
-  <si>
-    <t>fee</t>
-  </si>
-  <si>
-    <t>network</t>
-  </si>
-  <si>
-    <t>network issue</t>
-  </si>
-  <si>
-    <t>update request</t>
-  </si>
-  <si>
-    <t>address update</t>
-  </si>
-  <si>
-    <t>address</t>
-  </si>
-  <si>
-    <t>deducted incorrectly</t>
-  </si>
-  <si>
-    <t>incorrectly</t>
-  </si>
-  <si>
-    <t>incorrectly received</t>
-  </si>
-  <si>
-    <t>agent helpful</t>
-  </si>
-  <si>
-    <t>agent polite</t>
-  </si>
-  <si>
-    <t>agent resolved</t>
-  </si>
-  <si>
-    <t>clearly</t>
-  </si>
-  <si>
-    <t>great</t>
-  </si>
-  <si>
-    <t>great service</t>
-  </si>
-  <si>
-    <t>helpful</t>
-  </si>
-  <si>
-    <t>helpful professional</t>
-  </si>
-  <si>
-    <t>issue sorted</t>
-  </si>
-  <si>
-    <t>polite</t>
-  </si>
-  <si>
-    <t>polite explained</t>
-  </si>
-  <si>
-    <t>professional</t>
-  </si>
-  <si>
-    <t>quick</t>
-  </si>
-  <si>
-    <t>quick resolution</t>
-  </si>
-  <si>
-    <t>quickly</t>
-  </si>
-  <si>
-    <t>quickly polite</t>
-  </si>
-  <si>
-    <t>resolution</t>
-  </si>
-  <si>
-    <t>resolved</t>
-  </si>
-  <si>
-    <t>satisfied</t>
-  </si>
-  <si>
-    <t>satisfied agent</t>
-  </si>
-  <si>
-    <t>service</t>
   </si>
   <si>
     <t>sorted</t>
@@ -555,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -577,13 +583,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>1117</v>
+        <v>1099</v>
       </c>
       <c r="C2">
-        <v>1879</v>
+        <v>1793</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -591,13 +597,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>720</v>
+        <v>733</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -605,13 +611,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>705</v>
+        <v>681</v>
       </c>
       <c r="C4">
-        <v>1098</v>
+        <v>1062</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -619,13 +625,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>702</v>
+        <v>664</v>
       </c>
       <c r="C5">
-        <v>762</v>
+        <v>670</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -633,13 +639,13 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>700</v>
+        <v>649</v>
       </c>
       <c r="C6">
-        <v>646</v>
+        <v>761</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -647,13 +653,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>663</v>
+        <v>643</v>
       </c>
       <c r="C7">
-        <v>704</v>
+        <v>698</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -661,13 +667,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>546</v>
+        <v>566</v>
       </c>
       <c r="C8">
-        <v>368</v>
+        <v>636</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -675,13 +681,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>545</v>
+        <v>566</v>
       </c>
       <c r="C9">
-        <v>399</v>
+        <v>636</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -689,13 +695,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="C10">
-        <v>521</v>
+        <v>636</v>
       </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -703,13 +709,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>531</v>
+        <v>554</v>
       </c>
       <c r="C11">
-        <v>521</v>
+        <v>418</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -717,13 +723,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>514</v>
+        <v>478</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>533</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -731,13 +737,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>502</v>
+        <v>478</v>
       </c>
       <c r="C13">
-        <v>686</v>
+        <v>533</v>
       </c>
       <c r="D13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -745,13 +751,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>502</v>
+        <v>476</v>
       </c>
       <c r="C14">
-        <v>686</v>
+        <v>408</v>
       </c>
       <c r="D14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -759,13 +765,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>502</v>
+        <v>476</v>
       </c>
       <c r="C15">
-        <v>686</v>
+        <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -773,13 +779,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>473</v>
+        <v>399</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -787,13 +793,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C17">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -801,13 +807,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C18">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -815,13 +821,13 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C19">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -829,13 +835,13 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C20">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -843,13 +849,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -857,13 +863,13 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -871,13 +877,13 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="C23">
-        <v>325</v>
+        <v>0</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -885,13 +891,13 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -899,13 +905,13 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>355</v>
+        <v>339</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -913,13 +919,13 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>355</v>
+        <v>339</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -927,13 +933,13 @@
         <v>29</v>
       </c>
       <c r="B27">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -941,13 +947,13 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -955,13 +961,13 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="C29">
         <v>0</v>
       </c>
       <c r="D29" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -969,13 +975,13 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="C30">
         <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -983,13 +989,13 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="C31">
         <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -997,13 +1003,13 @@
         <v>34</v>
       </c>
       <c r="B32">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1011,13 +1017,13 @@
         <v>35</v>
       </c>
       <c r="B33">
-        <v>349</v>
+        <v>330</v>
       </c>
       <c r="C33">
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1025,13 +1031,13 @@
         <v>36</v>
       </c>
       <c r="B34">
-        <v>347</v>
+        <v>330</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1039,13 +1045,13 @@
         <v>37</v>
       </c>
       <c r="B35">
-        <v>347</v>
+        <v>330</v>
       </c>
       <c r="C35">
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1053,13 +1059,13 @@
         <v>38</v>
       </c>
       <c r="B36">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C36">
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1067,13 +1073,13 @@
         <v>39</v>
       </c>
       <c r="B37">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C37">
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1081,13 +1087,13 @@
         <v>40</v>
       </c>
       <c r="B38">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C38">
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -1098,10 +1104,10 @@
         <v>325</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>337</v>
       </c>
       <c r="D39" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -1112,10 +1118,10 @@
         <v>325</v>
       </c>
       <c r="C40">
-        <v>0</v>
+        <v>337</v>
       </c>
       <c r="D40" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -1126,10 +1132,10 @@
         <v>325</v>
       </c>
       <c r="C41">
-        <v>0</v>
+        <v>337</v>
       </c>
       <c r="D41" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1140,10 +1146,10 @@
         <v>0</v>
       </c>
       <c r="C42">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D42" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -1154,10 +1160,10 @@
         <v>0</v>
       </c>
       <c r="C43">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="D43" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1168,10 +1174,10 @@
         <v>0</v>
       </c>
       <c r="C44">
-        <v>497</v>
+        <v>452</v>
       </c>
       <c r="D44" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1182,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="C45">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="D45" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1196,10 +1202,10 @@
         <v>0</v>
       </c>
       <c r="C46">
-        <v>457</v>
+        <v>438</v>
       </c>
       <c r="D46" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1210,10 +1216,10 @@
         <v>0</v>
       </c>
       <c r="C47">
-        <v>457</v>
+        <v>438</v>
       </c>
       <c r="D47" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1224,10 +1230,10 @@
         <v>0</v>
       </c>
       <c r="C48">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D48" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -1238,10 +1244,10 @@
         <v>0</v>
       </c>
       <c r="C49">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D49" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -1252,10 +1258,10 @@
         <v>0</v>
       </c>
       <c r="C50">
-        <v>457</v>
+        <v>438</v>
       </c>
       <c r="D50" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1266,10 +1272,10 @@
         <v>0</v>
       </c>
       <c r="C51">
-        <v>951</v>
+        <v>336</v>
       </c>
       <c r="D51" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -1280,10 +1286,10 @@
         <v>0</v>
       </c>
       <c r="C52">
-        <v>454</v>
+        <v>914</v>
       </c>
       <c r="D52" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -1294,10 +1300,10 @@
         <v>0</v>
       </c>
       <c r="C53">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D53" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -1308,10 +1314,10 @@
         <v>0</v>
       </c>
       <c r="C54">
-        <v>414</v>
+        <v>462</v>
       </c>
       <c r="D54" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -1322,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="C55">
-        <v>414</v>
+        <v>510</v>
       </c>
       <c r="D55" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -1336,10 +1342,10 @@
         <v>0</v>
       </c>
       <c r="C56">
-        <v>497</v>
+        <v>510</v>
       </c>
       <c r="D56" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -1350,10 +1356,10 @@
         <v>0</v>
       </c>
       <c r="C57">
-        <v>497</v>
+        <v>452</v>
       </c>
       <c r="D57" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -1364,10 +1370,10 @@
         <v>0</v>
       </c>
       <c r="C58">
-        <v>496</v>
+        <v>452</v>
       </c>
       <c r="D58" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -1378,10 +1384,10 @@
         <v>0</v>
       </c>
       <c r="C59">
-        <v>580</v>
+        <v>618</v>
       </c>
       <c r="D59" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -1392,10 +1398,10 @@
         <v>0</v>
       </c>
       <c r="C60">
-        <v>476</v>
+        <v>534</v>
       </c>
       <c r="D60" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -1406,10 +1412,10 @@
         <v>0</v>
       </c>
       <c r="C61">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D61" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -1420,10 +1426,10 @@
         <v>0</v>
       </c>
       <c r="C62">
-        <v>523</v>
+        <v>462</v>
       </c>
       <c r="D62" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -1434,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="C63">
-        <v>457</v>
+        <v>508</v>
       </c>
       <c r="D63" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -1448,10 +1454,38 @@
         <v>0</v>
       </c>
       <c r="C64">
-        <v>414</v>
+        <v>337</v>
       </c>
       <c r="D64" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" t="s">
         <v>67</v>
+      </c>
+      <c r="B65">
+        <v>0</v>
+      </c>
+      <c r="C65">
+        <v>438</v>
+      </c>
+      <c r="D65" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
+      </c>
+      <c r="C66">
+        <v>510</v>
+      </c>
+      <c r="D66" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix agent_name realism: no index suffix, no repeated name parts across the roster
build_agent_roster() appended a "(i+1)" index to every agent_name purely
to dodge collisions in a small 20x10 first/last name grid - that index
leaked into the actual data column, which a real agent-name field would
never carry. Expanded both name pools to 30 entries each and sample first
and last names independently without replacement, so every one of the 24
agents gets a genuinely unique first name AND unique last name, not just
a unique full-name combination. Regenerated input/intermediate/final
output and updated narration_script.md's quoted numbers to match the new
(expected) random-sequence drift.
</commit_message>
<xml_diff>
--- a/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
+++ b/usecase1_csat_nlp_rootcause/intermediate/intermediate_dictionary_bootstrap_terms.xlsx
@@ -37,12 +37,12 @@
     <t>time</t>
   </si>
   <si>
+    <t>honestly</t>
+  </si>
+  <si>
     <t>simply</t>
   </si>
   <si>
-    <t>honestly</t>
-  </si>
-  <si>
     <t>going lie</t>
   </si>
   <si>
@@ -55,39 +55,39 @@
     <t>say</t>
   </si>
   <si>
+    <t>really</t>
+  </si>
+  <si>
+    <t>really frustrated</t>
+  </si>
+  <si>
+    <t>frustrated</t>
+  </si>
+  <si>
+    <t>far</t>
+  </si>
+  <si>
+    <t>fixed</t>
+  </si>
+  <si>
+    <t>change</t>
+  </si>
+  <si>
+    <t>acceptable</t>
+  </si>
+  <si>
+    <t>far acceptable</t>
+  </si>
+  <si>
+    <t>honest</t>
+  </si>
+  <si>
     <t>simply good</t>
   </si>
   <si>
     <t>good</t>
   </si>
   <si>
-    <t>far</t>
-  </si>
-  <si>
-    <t>really</t>
-  </si>
-  <si>
-    <t>really frustrated</t>
-  </si>
-  <si>
-    <t>frustrated</t>
-  </si>
-  <si>
-    <t>fixed</t>
-  </si>
-  <si>
-    <t>honest</t>
-  </si>
-  <si>
-    <t>acceptable</t>
-  </si>
-  <si>
-    <t>far acceptable</t>
-  </si>
-  <si>
-    <t>change</t>
-  </si>
-  <si>
     <t>frustrating experience</t>
   </si>
   <si>
@@ -100,85 +100,91 @@
     <t>experience overall</t>
   </si>
   <si>
+    <t>experience expected</t>
+  </si>
+  <si>
+    <t>expected</t>
+  </si>
+  <si>
+    <t>needs change</t>
+  </si>
+  <si>
     <t>account</t>
   </si>
   <si>
-    <t>experience expected</t>
-  </si>
-  <si>
-    <t>expected</t>
-  </si>
-  <si>
     <t>fixed soon</t>
   </si>
   <si>
+    <t>soon</t>
+  </si>
+  <si>
     <t>needs fixed</t>
   </si>
   <si>
-    <t>soon</t>
-  </si>
-  <si>
-    <t>needs change</t>
+    <t>just</t>
+  </si>
+  <si>
+    <t>month</t>
   </si>
   <si>
     <t>got</t>
   </si>
   <si>
-    <t>just</t>
-  </si>
-  <si>
-    <t>month</t>
-  </si>
-  <si>
     <t>payment</t>
   </si>
   <si>
+    <t>agent</t>
+  </si>
+  <si>
     <t>told</t>
   </si>
   <si>
-    <t>agent</t>
+    <t>team</t>
   </si>
   <si>
     <t>ve</t>
   </si>
   <si>
+    <t>plan</t>
+  </si>
+  <si>
+    <t>charge</t>
+  </si>
+  <si>
     <t>hi</t>
   </si>
   <si>
-    <t>team</t>
-  </si>
-  <si>
-    <t>plan</t>
-  </si>
-  <si>
-    <t>charge</t>
+    <t>don</t>
   </si>
   <si>
     <t>actually</t>
   </si>
   <si>
-    <t>don</t>
-  </si>
-  <si>
     <t>support</t>
   </si>
   <si>
+    <t>twice</t>
+  </si>
+  <si>
+    <t>tax</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
     <t>roaming</t>
   </si>
   <si>
-    <t>twice</t>
-  </si>
-  <si>
-    <t>tax</t>
+    <t>given</t>
   </si>
   <si>
     <t>issue</t>
   </si>
   <si>
-    <t>days</t>
-  </si>
-  <si>
-    <t>given</t>
+    <t>connection</t>
+  </si>
+  <si>
+    <t>times</t>
   </si>
   <si>
     <t>refund</t>
@@ -190,277 +196,358 @@
     <t>fee</t>
   </si>
   <si>
-    <t>times</t>
-  </si>
-  <si>
-    <t>connection</t>
-  </si>
-  <si>
     <t>completely</t>
   </si>
   <si>
+    <t>charged</t>
+  </si>
+  <si>
+    <t>shows</t>
+  </si>
+  <si>
+    <t>paid</t>
+  </si>
+  <si>
+    <t>zero</t>
+  </si>
+  <si>
     <t>late</t>
   </si>
   <si>
     <t>different</t>
   </si>
   <si>
-    <t>shows</t>
-  </si>
-  <si>
-    <t>zero</t>
+    <t>problem</t>
+  </si>
+  <si>
+    <t>keeps</t>
+  </si>
+  <si>
+    <t>doesn</t>
+  </si>
+  <si>
+    <t>billed</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
   <si>
     <t>service</t>
   </si>
   <si>
-    <t>paid</t>
-  </si>
-  <si>
-    <t>charged</t>
-  </si>
-  <si>
-    <t>billed</t>
-  </si>
-  <si>
-    <t>doesn</t>
-  </si>
-  <si>
-    <t>new</t>
-  </si>
-  <si>
-    <t>problem</t>
-  </si>
-  <si>
-    <t>keeps</t>
+    <t>entire</t>
   </si>
   <si>
     <t>pack</t>
   </si>
   <si>
+    <t>international</t>
+  </si>
+  <si>
     <t>came</t>
   </si>
   <si>
-    <t>entire</t>
+    <t>explain</t>
   </si>
   <si>
     <t>line</t>
   </si>
   <si>
-    <t>explain</t>
-  </si>
-  <si>
-    <t>international</t>
-  </si>
-  <si>
     <t>promised</t>
   </si>
   <si>
+    <t>went</t>
+  </si>
+  <si>
     <t>like</t>
   </si>
   <si>
+    <t>don understand</t>
+  </si>
+  <si>
+    <t>understand</t>
+  </si>
+  <si>
+    <t>thing</t>
+  </si>
+  <si>
     <t>concern</t>
   </si>
   <si>
-    <t>went</t>
-  </si>
-  <si>
-    <t>thing</t>
+    <t>roaming charge</t>
+  </si>
+  <si>
+    <t>cycle</t>
+  </si>
+  <si>
+    <t>supposedly</t>
+  </si>
+  <si>
+    <t>penalty</t>
+  </si>
+  <si>
+    <t>hi team</t>
+  </si>
+  <si>
+    <t>asked</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>match</t>
+  </si>
+  <si>
+    <t>genuinely</t>
+  </si>
+  <si>
+    <t>hello</t>
   </si>
   <si>
     <t>late fee</t>
   </si>
   <si>
-    <t>genuinely</t>
+    <t>second</t>
+  </si>
+  <si>
+    <t>signal</t>
   </si>
   <si>
     <t>escalated</t>
   </si>
   <si>
-    <t>asked</t>
-  </si>
-  <si>
-    <t>cycle</t>
-  </si>
-  <si>
-    <t>don understand</t>
-  </si>
-  <si>
-    <t>understand</t>
-  </si>
-  <si>
-    <t>roaming charge</t>
-  </si>
-  <si>
-    <t>hi team</t>
+    <t>balance</t>
+  </si>
+  <si>
+    <t>dear support</t>
+  </si>
+  <si>
+    <t>support team</t>
+  </si>
+  <si>
+    <t>waiting</t>
+  </si>
+  <si>
+    <t>dear</t>
+  </si>
+  <si>
+    <t>specifically</t>
+  </si>
+  <si>
+    <t>despite</t>
+  </si>
+  <si>
+    <t>hold</t>
   </si>
   <si>
     <t>happened</t>
   </si>
   <si>
-    <t>penalty</t>
-  </si>
-  <si>
-    <t>waiting</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>hello</t>
-  </si>
-  <si>
-    <t>supposedly</t>
-  </si>
-  <si>
-    <t>home</t>
-  </si>
-  <si>
-    <t>match</t>
-  </si>
-  <si>
-    <t>signal</t>
+    <t>ago</t>
+  </si>
+  <si>
+    <t>speed</t>
+  </si>
+  <si>
+    <t>item</t>
+  </si>
+  <si>
+    <t>line item</t>
+  </si>
+  <si>
+    <t>sitting</t>
+  </si>
+  <si>
+    <t>statement</t>
   </si>
   <si>
     <t>single</t>
   </si>
   <si>
-    <t>despite</t>
-  </si>
-  <si>
-    <t>specifically</t>
-  </si>
-  <si>
-    <t>item</t>
-  </si>
-  <si>
-    <t>line item</t>
-  </si>
-  <si>
-    <t>balance</t>
-  </si>
-  <si>
-    <t>statement</t>
-  </si>
-  <si>
-    <t>dear support</t>
+    <t>getting</t>
+  </si>
+  <si>
+    <t>left</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>minutes</t>
+  </si>
+  <si>
+    <t>answer</t>
+  </si>
+  <si>
+    <t>doesn match</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>passed</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>later</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>calls</t>
   </si>
   <si>
     <t>account genuinely</t>
   </si>
   <si>
-    <t>sitting</t>
-  </si>
-  <si>
-    <t>dear</t>
-  </si>
-  <si>
-    <t>ago</t>
-  </si>
-  <si>
-    <t>support team</t>
-  </si>
-  <si>
-    <t>hold</t>
-  </si>
-  <si>
-    <t>speed</t>
-  </si>
-  <si>
-    <t>left</t>
+    <t>make</t>
+  </si>
+  <si>
+    <t>invoice</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t>changing</t>
   </si>
   <si>
     <t>request</t>
   </si>
   <si>
-    <t>second</t>
-  </si>
-  <si>
-    <t>minutes</t>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>money</t>
   </si>
   <si>
     <t>start</t>
   </si>
   <si>
-    <t>answer</t>
-  </si>
-  <si>
-    <t>phone</t>
-  </si>
-  <si>
-    <t>area</t>
-  </si>
-  <si>
-    <t>getting</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>explanation</t>
-  </si>
-  <si>
-    <t>invoice</t>
-  </si>
-  <si>
-    <t>make</t>
-  </si>
-  <si>
-    <t>doesn match</t>
-  </si>
-  <si>
-    <t>calls</t>
+    <t>installation</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>outage</t>
+  </si>
+  <si>
+    <t>resolved</t>
   </si>
   <si>
     <t>shouldn</t>
   </si>
   <si>
-    <t>passed</t>
+    <t>turned</t>
+  </si>
+  <si>
+    <t>spoke</t>
+  </si>
+  <si>
+    <t>right</t>
+  </si>
+  <si>
+    <t>explained</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>department</t>
   </si>
   <si>
     <t>explaining</t>
   </si>
   <si>
-    <t>spoke</t>
-  </si>
-  <si>
-    <t>turned</t>
-  </si>
-  <si>
-    <t>later</t>
-  </si>
-  <si>
-    <t>cut</t>
-  </si>
-  <si>
-    <t>money</t>
+    <t>complete</t>
   </si>
   <si>
     <t>add</t>
   </si>
   <si>
-    <t>count</t>
+    <t>called</t>
+  </si>
+  <si>
+    <t>instead</t>
+  </si>
+  <si>
+    <t>gotten</t>
+  </si>
+  <si>
+    <t>second time</t>
+  </si>
+  <si>
+    <t>hours</t>
+  </si>
+  <si>
+    <t>used</t>
+  </si>
+  <si>
+    <t>disconnected</t>
+  </si>
+  <si>
+    <t>got disconnected</t>
+  </si>
+  <si>
+    <t>charge account</t>
+  </si>
+  <si>
+    <t>traveled</t>
   </si>
   <si>
     <t>case</t>
   </si>
   <si>
-    <t>changing</t>
-  </si>
-  <si>
-    <t>outage</t>
-  </si>
-  <si>
-    <t>right</t>
-  </si>
-  <si>
-    <t>hours</t>
+    <t>contacting</t>
+  </si>
+  <si>
+    <t>international charge</t>
+  </si>
+  <si>
+    <t>account haven</t>
+  </si>
+  <si>
+    <t>haven</t>
+  </si>
+  <si>
+    <t>haven traveled</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>traveled months</t>
+  </si>
+  <si>
+    <t>callback</t>
+  </si>
+  <si>
+    <t>dropped</t>
+  </si>
+  <si>
+    <t>slow</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>near</t>
+  </si>
+  <si>
+    <t>week</t>
   </si>
   <si>
     <t>makes</t>
   </si>
   <si>
-    <t>clear</t>
+    <t>tried</t>
   </si>
   <si>
     <t>sense</t>
@@ -469,163 +556,76 @@
     <t>makes sense</t>
   </si>
   <si>
-    <t>complete</t>
+    <t>charge signed</t>
+  </si>
+  <si>
+    <t>signed</t>
+  </si>
+  <si>
+    <t>idea</t>
+  </si>
+  <si>
+    <t>international roaming</t>
+  </si>
+  <si>
+    <t>reach</t>
+  </si>
+  <si>
+    <t>explain international</t>
+  </si>
+  <si>
+    <t>past</t>
+  </si>
+  <si>
+    <t>person</t>
+  </si>
+  <si>
+    <t>data speed</t>
+  </si>
+  <si>
+    <t>speed plan</t>
   </si>
   <si>
     <t>showed</t>
   </si>
   <si>
-    <t>contacting</t>
-  </si>
-  <si>
-    <t>got disconnected</t>
-  </si>
-  <si>
-    <t>disconnected</t>
-  </si>
-  <si>
-    <t>instead</t>
-  </si>
-  <si>
-    <t>installation</t>
-  </si>
-  <si>
-    <t>gotten</t>
+    <t>recharge</t>
+  </si>
+  <si>
+    <t>mid</t>
+  </si>
+  <si>
+    <t>keeps changing</t>
+  </si>
+  <si>
+    <t>gst</t>
   </si>
   <si>
     <t>gone</t>
   </si>
   <si>
-    <t>reason</t>
-  </si>
-  <si>
-    <t>used</t>
-  </si>
-  <si>
-    <t>called</t>
-  </si>
-  <si>
-    <t>callback</t>
-  </si>
-  <si>
-    <t>slow</t>
-  </si>
-  <si>
-    <t>haven</t>
-  </si>
-  <si>
-    <t>haven traveled</t>
-  </si>
-  <si>
-    <t>charge account</t>
-  </si>
-  <si>
-    <t>traveled</t>
-  </si>
-  <si>
-    <t>traveled months</t>
-  </si>
-  <si>
-    <t>international charge</t>
-  </si>
-  <si>
-    <t>resolved</t>
-  </si>
-  <si>
-    <t>account haven</t>
-  </si>
-  <si>
-    <t>months</t>
-  </si>
-  <si>
-    <t>week</t>
-  </si>
-  <si>
-    <t>speed plan</t>
-  </si>
-  <si>
-    <t>explained</t>
-  </si>
-  <si>
-    <t>apparently</t>
-  </si>
-  <si>
-    <t>dropped</t>
-  </si>
-  <si>
-    <t>tried</t>
-  </si>
-  <si>
-    <t>need</t>
-  </si>
-  <si>
-    <t>department</t>
-  </si>
-  <si>
-    <t>past</t>
-  </si>
-  <si>
-    <t>reach</t>
-  </si>
-  <si>
-    <t>idea</t>
-  </si>
-  <si>
-    <t>asked escalated</t>
-  </si>
-  <si>
-    <t>second time</t>
-  </si>
-  <si>
-    <t>near</t>
-  </si>
-  <si>
-    <t>minute</t>
+    <t>gst component</t>
   </si>
   <si>
     <t>exact</t>
   </si>
   <si>
-    <t>data speed</t>
-  </si>
-  <si>
-    <t>explain international</t>
-  </si>
-  <si>
-    <t>charge signed</t>
-  </si>
-  <si>
-    <t>signed</t>
-  </si>
-  <si>
-    <t>warning</t>
-  </si>
-  <si>
-    <t>international roaming</t>
-  </si>
-  <si>
-    <t>mid</t>
-  </si>
-  <si>
-    <t>person</t>
-  </si>
-  <si>
-    <t>fee paid</t>
-  </si>
-  <si>
-    <t>recharge</t>
-  </si>
-  <si>
-    <t>outside</t>
-  </si>
-  <si>
-    <t>paid date</t>
+    <t>documents</t>
   </si>
   <si>
     <t>time month</t>
   </si>
   <si>
-    <t>followed</t>
+    <t>changing month</t>
+  </si>
+  <si>
+    <t>component keeps</t>
+  </si>
+  <si>
+    <t>component</t>
+  </si>
+  <si>
+    <t>validity</t>
   </si>
   <si>
     <t>sorted single</t>
@@ -1282,7 +1282,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>668</v>
+        <v>695</v>
       </c>
       <c r="C2">
         <v>565</v>
@@ -1296,10 +1296,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="C3">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D3" t="s">
         <v>303</v>
@@ -1310,10 +1310,10 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="C4">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="D4" t="s">
         <v>303</v>
@@ -1324,10 +1324,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C5">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D5" t="s">
         <v>303</v>
@@ -1338,10 +1338,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>452</v>
+        <v>430</v>
       </c>
       <c r="C6">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="D6" t="s">
         <v>303</v>
@@ -1352,10 +1352,10 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C7">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D7" t="s">
         <v>303</v>
@@ -1366,10 +1366,10 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C8">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D8" t="s">
         <v>303</v>
@@ -1380,10 +1380,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C9">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D9" t="s">
         <v>303</v>
@@ -1394,10 +1394,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="C10">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D10" t="s">
         <v>303</v>
@@ -1408,13 +1408,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="C11">
-        <v>144</v>
+        <v>529</v>
       </c>
       <c r="D11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1422,13 +1422,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="C12">
-        <v>330</v>
+        <v>152</v>
       </c>
       <c r="D12" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1436,7 +1436,7 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="C13">
         <v>152</v>
@@ -1450,13 +1450,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="C14">
-        <v>531</v>
+        <v>153</v>
       </c>
       <c r="D14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1464,10 +1464,10 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C15">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="D15" t="s">
         <v>303</v>
@@ -1478,10 +1478,10 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="C16">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
         <v>303</v>
@@ -1492,10 +1492,10 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="C17">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D17" t="s">
         <v>303</v>
@@ -1506,10 +1506,10 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="C18">
-        <v>171</v>
+        <v>140</v>
       </c>
       <c r="D18" t="s">
         <v>303</v>
@@ -1520,10 +1520,10 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C19">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="D19" t="s">
         <v>303</v>
@@ -1534,10 +1534,10 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C20">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D20" t="s">
         <v>303</v>
@@ -1548,13 +1548,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C21">
-        <v>115</v>
+        <v>326</v>
       </c>
       <c r="D21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1562,10 +1562,10 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>336</v>
+        <v>353</v>
       </c>
       <c r="C22">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D22" t="s">
         <v>303</v>
@@ -1576,10 +1576,10 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>336</v>
+        <v>353</v>
       </c>
       <c r="C23">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D23" t="s">
         <v>303</v>
@@ -1590,10 +1590,10 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>336</v>
+        <v>353</v>
       </c>
       <c r="C24">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D24" t="s">
         <v>303</v>
@@ -1604,10 +1604,10 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>336</v>
+        <v>353</v>
       </c>
       <c r="C25">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D25" t="s">
         <v>303</v>
@@ -1618,10 +1618,10 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="C26">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
         <v>303</v>
@@ -1632,13 +1632,13 @@
         <v>29</v>
       </c>
       <c r="B27">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C27">
-        <v>140</v>
+        <v>234</v>
       </c>
       <c r="D27" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1646,13 +1646,13 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C28">
-        <v>243</v>
+        <v>110</v>
       </c>
       <c r="D28" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1660,10 +1660,10 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C29">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
         <v>303</v>
@@ -1674,10 +1674,10 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C30">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D30" t="s">
         <v>303</v>
@@ -1688,10 +1688,10 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C31">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D31" t="s">
         <v>303</v>
@@ -1702,10 +1702,10 @@
         <v>34</v>
       </c>
       <c r="B32">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C32">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D32" t="s">
         <v>303</v>
@@ -1719,7 +1719,7 @@
         <v>269</v>
       </c>
       <c r="C33">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="D33" t="s">
         <v>303</v>
@@ -1730,10 +1730,10 @@
         <v>36</v>
       </c>
       <c r="B34">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C34">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D34" t="s">
         <v>303</v>
@@ -1744,10 +1744,10 @@
         <v>37</v>
       </c>
       <c r="B35">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C35">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D35" t="s">
         <v>303</v>
@@ -1758,10 +1758,10 @@
         <v>38</v>
       </c>
       <c r="B36">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C36">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D36" t="s">
         <v>303</v>
@@ -1772,13 +1772,13 @@
         <v>39</v>
       </c>
       <c r="B37">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C37">
-        <v>107</v>
+        <v>403</v>
       </c>
       <c r="D37" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1786,13 +1786,13 @@
         <v>40</v>
       </c>
       <c r="B38">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C38">
-        <v>396</v>
+        <v>106</v>
       </c>
       <c r="D38" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -1800,13 +1800,13 @@
         <v>41</v>
       </c>
       <c r="B39">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C39">
-        <v>88</v>
+        <v>309</v>
       </c>
       <c r="D39" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -1814,13 +1814,13 @@
         <v>42</v>
       </c>
       <c r="B40">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C40">
-        <v>189</v>
+        <v>93</v>
       </c>
       <c r="D40" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -1828,13 +1828,13 @@
         <v>43</v>
       </c>
       <c r="B41">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C41">
-        <v>310</v>
+        <v>81</v>
       </c>
       <c r="D41" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1842,10 +1842,10 @@
         <v>44</v>
       </c>
       <c r="B42">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C42">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="D42" t="s">
         <v>303</v>
@@ -1856,13 +1856,13 @@
         <v>45</v>
       </c>
       <c r="B43">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C43">
-        <v>66</v>
+        <v>185</v>
       </c>
       <c r="D43" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1870,10 +1870,10 @@
         <v>46</v>
       </c>
       <c r="B44">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C44">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D44" t="s">
         <v>303</v>
@@ -1884,7 +1884,7 @@
         <v>47</v>
       </c>
       <c r="B45">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C45">
         <v>81</v>
@@ -1898,10 +1898,10 @@
         <v>48</v>
       </c>
       <c r="B46">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C46">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D46" t="s">
         <v>302</v>
@@ -1912,10 +1912,10 @@
         <v>49</v>
       </c>
       <c r="B47">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C47">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="D47" t="s">
         <v>303</v>
@@ -1926,10 +1926,10 @@
         <v>50</v>
       </c>
       <c r="B48">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C48">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="D48" t="s">
         <v>303</v>
@@ -1940,10 +1940,10 @@
         <v>51</v>
       </c>
       <c r="B49">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C49">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D49" t="s">
         <v>303</v>
@@ -1954,13 +1954,13 @@
         <v>52</v>
       </c>
       <c r="B50">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C50">
-        <v>164</v>
+        <v>66</v>
       </c>
       <c r="D50" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1968,10 +1968,10 @@
         <v>53</v>
       </c>
       <c r="B51">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C51">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="D51" t="s">
         <v>303</v>
@@ -1982,13 +1982,13 @@
         <v>54</v>
       </c>
       <c r="B52">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C52">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="D52" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -1996,10 +1996,10 @@
         <v>55</v>
       </c>
       <c r="B53">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C53">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="D53" t="s">
         <v>303</v>
@@ -2010,10 +2010,10 @@
         <v>56</v>
       </c>
       <c r="B54">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C54">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D54" t="s">
         <v>303</v>
@@ -2024,10 +2024,10 @@
         <v>57</v>
       </c>
       <c r="B55">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C55">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="D55" t="s">
         <v>303</v>
@@ -2038,10 +2038,10 @@
         <v>58</v>
       </c>
       <c r="B56">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C56">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D56" t="s">
         <v>303</v>
@@ -2052,10 +2052,10 @@
         <v>59</v>
       </c>
       <c r="B57">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C57">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D57" t="s">
         <v>303</v>
@@ -2066,10 +2066,10 @@
         <v>60</v>
       </c>
       <c r="B58">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C58">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D58" t="s">
         <v>303</v>
@@ -2080,10 +2080,10 @@
         <v>61</v>
       </c>
       <c r="B59">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C59">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D59" t="s">
         <v>303</v>
@@ -2094,10 +2094,10 @@
         <v>62</v>
       </c>
       <c r="B60">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C60">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D60" t="s">
         <v>303</v>
@@ -2111,7 +2111,7 @@
         <v>144</v>
       </c>
       <c r="C61">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D61" t="s">
         <v>303</v>
@@ -2122,10 +2122,10 @@
         <v>64</v>
       </c>
       <c r="B62">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C62">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D62" t="s">
         <v>303</v>
@@ -2136,13 +2136,13 @@
         <v>65</v>
       </c>
       <c r="B63">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C63">
-        <v>243</v>
+        <v>68</v>
       </c>
       <c r="D63" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2150,10 +2150,10 @@
         <v>66</v>
       </c>
       <c r="B64">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C64">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D64" t="s">
         <v>303</v>
@@ -2164,10 +2164,10 @@
         <v>67</v>
       </c>
       <c r="B65">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C65">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="D65" t="s">
         <v>303</v>
@@ -2178,10 +2178,10 @@
         <v>68</v>
       </c>
       <c r="B66">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C66">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D66" t="s">
         <v>303</v>
@@ -2192,10 +2192,10 @@
         <v>69</v>
       </c>
       <c r="B67">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C67">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D67" t="s">
         <v>303</v>
@@ -2206,10 +2206,10 @@
         <v>70</v>
       </c>
       <c r="B68">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="D68" t="s">
         <v>303</v>
@@ -2220,10 +2220,10 @@
         <v>71</v>
       </c>
       <c r="B69">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C69">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D69" t="s">
         <v>303</v>
@@ -2234,13 +2234,13 @@
         <v>72</v>
       </c>
       <c r="B70">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C70">
-        <v>49</v>
+        <v>245</v>
       </c>
       <c r="D70" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2248,10 +2248,10 @@
         <v>73</v>
       </c>
       <c r="B71">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C71">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D71" t="s">
         <v>303</v>
@@ -2262,10 +2262,10 @@
         <v>74</v>
       </c>
       <c r="B72">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C72">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D72" t="s">
         <v>303</v>
@@ -2276,10 +2276,10 @@
         <v>75</v>
       </c>
       <c r="B73">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C73">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="D73" t="s">
         <v>303</v>
@@ -2290,7 +2290,7 @@
         <v>76</v>
       </c>
       <c r="B74">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C74">
         <v>46</v>
@@ -2307,7 +2307,7 @@
         <v>123</v>
       </c>
       <c r="C75">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D75" t="s">
         <v>303</v>
@@ -2318,10 +2318,10 @@
         <v>78</v>
       </c>
       <c r="B76">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C76">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D76" t="s">
         <v>303</v>
@@ -2332,10 +2332,10 @@
         <v>79</v>
       </c>
       <c r="B77">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C77">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="D77" t="s">
         <v>302</v>
@@ -2346,13 +2346,13 @@
         <v>80</v>
       </c>
       <c r="B78">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C78">
-        <v>40</v>
+        <v>152</v>
       </c>
       <c r="D78" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -2360,13 +2360,13 @@
         <v>81</v>
       </c>
       <c r="B79">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C79">
-        <v>298</v>
+        <v>43</v>
       </c>
       <c r="D79" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -2377,10 +2377,10 @@
         <v>113</v>
       </c>
       <c r="C80">
-        <v>154</v>
+        <v>42</v>
       </c>
       <c r="D80" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -2388,10 +2388,10 @@
         <v>83</v>
       </c>
       <c r="B81">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C81">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="D81" t="s">
         <v>303</v>
@@ -2402,10 +2402,10 @@
         <v>84</v>
       </c>
       <c r="B82">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C82">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D82" t="s">
         <v>303</v>
@@ -2419,10 +2419,10 @@
         <v>107</v>
       </c>
       <c r="C83">
-        <v>157</v>
+        <v>291</v>
       </c>
       <c r="D83" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -2430,10 +2430,10 @@
         <v>86</v>
       </c>
       <c r="B84">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C84">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="D84" t="s">
         <v>303</v>
@@ -2444,7 +2444,7 @@
         <v>87</v>
       </c>
       <c r="B85">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C85">
         <v>40</v>
@@ -2472,10 +2472,10 @@
         <v>89</v>
       </c>
       <c r="B87">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C87">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="D87" t="s">
         <v>303</v>
@@ -2486,13 +2486,13 @@
         <v>90</v>
       </c>
       <c r="B88">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C88">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="D88" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -2500,7 +2500,7 @@
         <v>91</v>
       </c>
       <c r="B89">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -2514,13 +2514,13 @@
         <v>92</v>
       </c>
       <c r="B90">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C90">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="D90" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -2542,7 +2542,7 @@
         <v>94</v>
       </c>
       <c r="B92">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -2556,13 +2556,13 @@
         <v>95</v>
       </c>
       <c r="B93">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C93">
-        <v>41</v>
+        <v>149</v>
       </c>
       <c r="D93" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -2570,13 +2570,13 @@
         <v>96</v>
       </c>
       <c r="B94">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C94">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="D94" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -2584,13 +2584,13 @@
         <v>97</v>
       </c>
       <c r="B95">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C95">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="D95" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -2598,7 +2598,7 @@
         <v>98</v>
       </c>
       <c r="B96">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C96">
         <v>0</v>
@@ -2612,10 +2612,10 @@
         <v>99</v>
       </c>
       <c r="B97">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C97">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D97" t="s">
         <v>303</v>
@@ -2626,10 +2626,10 @@
         <v>100</v>
       </c>
       <c r="B98">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C98">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D98" t="s">
         <v>303</v>
@@ -2640,10 +2640,10 @@
         <v>101</v>
       </c>
       <c r="B99">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C99">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D99" t="s">
         <v>303</v>
@@ -2654,10 +2654,10 @@
         <v>102</v>
       </c>
       <c r="B100">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C100">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="D100" t="s">
         <v>302</v>
@@ -2668,13 +2668,13 @@
         <v>103</v>
       </c>
       <c r="B101">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C101">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D101" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -2682,10 +2682,10 @@
         <v>104</v>
       </c>
       <c r="B102">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C102">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="D102" t="s">
         <v>303</v>
@@ -2699,10 +2699,10 @@
         <v>91</v>
       </c>
       <c r="C103">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D103" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -2710,7 +2710,7 @@
         <v>106</v>
       </c>
       <c r="B104">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C104">
         <v>0</v>
@@ -2727,7 +2727,7 @@
         <v>90</v>
       </c>
       <c r="C105">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D105" t="s">
         <v>303</v>
@@ -2741,7 +2741,7 @@
         <v>90</v>
       </c>
       <c r="C106">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D106" t="s">
         <v>303</v>
@@ -2752,13 +2752,13 @@
         <v>109</v>
       </c>
       <c r="B107">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C107">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="D107" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -2769,7 +2769,7 @@
         <v>89</v>
       </c>
       <c r="C108">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="D108" t="s">
         <v>303</v>
@@ -2794,13 +2794,13 @@
         <v>112</v>
       </c>
       <c r="B110">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C110">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -2808,7 +2808,7 @@
         <v>113</v>
       </c>
       <c r="B111">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -2822,13 +2822,13 @@
         <v>114</v>
       </c>
       <c r="B112">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C112">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="D112" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -2836,10 +2836,10 @@
         <v>115</v>
       </c>
       <c r="B113">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C113">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D113" t="s">
         <v>303</v>
@@ -2850,13 +2850,13 @@
         <v>116</v>
       </c>
       <c r="B114">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C114">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="D114" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -2864,7 +2864,7 @@
         <v>117</v>
       </c>
       <c r="B115">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -2878,13 +2878,13 @@
         <v>118</v>
       </c>
       <c r="B116">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C116">
-        <v>137</v>
+        <v>0</v>
       </c>
       <c r="D116" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -2906,10 +2906,10 @@
         <v>120</v>
       </c>
       <c r="B118">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C118">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D118" t="s">
         <v>304</v>
@@ -2923,10 +2923,10 @@
         <v>82</v>
       </c>
       <c r="C119">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="D119" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -2934,7 +2934,7 @@
         <v>122</v>
       </c>
       <c r="B120">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -2948,7 +2948,7 @@
         <v>123</v>
       </c>
       <c r="B121">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -2962,7 +2962,7 @@
         <v>124</v>
       </c>
       <c r="B122">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -2990,7 +2990,7 @@
         <v>126</v>
       </c>
       <c r="B124">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -3004,7 +3004,7 @@
         <v>127</v>
       </c>
       <c r="B125">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C125">
         <v>0</v>
@@ -3032,10 +3032,10 @@
         <v>129</v>
       </c>
       <c r="B127">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C127">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D127" t="s">
         <v>303</v>
@@ -3046,7 +3046,7 @@
         <v>130</v>
       </c>
       <c r="B128">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C128">
         <v>0</v>
@@ -3060,7 +3060,7 @@
         <v>131</v>
       </c>
       <c r="B129">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -3105,10 +3105,10 @@
         <v>76</v>
       </c>
       <c r="C132">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="D132" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -3119,7 +3119,7 @@
         <v>76</v>
       </c>
       <c r="C133">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D133" t="s">
         <v>303</v>
@@ -3130,7 +3130,7 @@
         <v>136</v>
       </c>
       <c r="B134">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -3144,13 +3144,13 @@
         <v>137</v>
       </c>
       <c r="B135">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C135">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D135" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -3158,10 +3158,10 @@
         <v>138</v>
       </c>
       <c r="B136">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C136">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D136" t="s">
         <v>303</v>
@@ -3172,10 +3172,10 @@
         <v>139</v>
       </c>
       <c r="B137">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C137">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="D137" t="s">
         <v>303</v>
@@ -3186,7 +3186,7 @@
         <v>140</v>
       </c>
       <c r="B138">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -3200,13 +3200,13 @@
         <v>141</v>
       </c>
       <c r="B139">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="D139" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -3214,7 +3214,7 @@
         <v>142</v>
       </c>
       <c r="B140">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -3228,7 +3228,7 @@
         <v>143</v>
       </c>
       <c r="B141">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -3242,7 +3242,7 @@
         <v>144</v>
       </c>
       <c r="B142">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -3256,7 +3256,7 @@
         <v>145</v>
       </c>
       <c r="B143">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C143">
         <v>0</v>
@@ -3270,13 +3270,13 @@
         <v>146</v>
       </c>
       <c r="B144">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C144">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="D144" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -3284,7 +3284,7 @@
         <v>147</v>
       </c>
       <c r="B145">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -3298,7 +3298,7 @@
         <v>148</v>
       </c>
       <c r="B146">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -3312,7 +3312,7 @@
         <v>149</v>
       </c>
       <c r="B147">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -3326,7 +3326,7 @@
         <v>150</v>
       </c>
       <c r="B148">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C148">
         <v>0</v>
@@ -3340,7 +3340,7 @@
         <v>151</v>
       </c>
       <c r="B149">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -3354,7 +3354,7 @@
         <v>152</v>
       </c>
       <c r="B150">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -3396,7 +3396,7 @@
         <v>155</v>
       </c>
       <c r="B153">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -3424,10 +3424,10 @@
         <v>157</v>
       </c>
       <c r="B155">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C155">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D155" t="s">
         <v>303</v>
@@ -3438,7 +3438,7 @@
         <v>158</v>
       </c>
       <c r="B156">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -3466,7 +3466,7 @@
         <v>160</v>
       </c>
       <c r="B158">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3480,7 +3480,7 @@
         <v>161</v>
       </c>
       <c r="B159">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -3536,7 +3536,7 @@
         <v>165</v>
       </c>
       <c r="B163">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -3550,7 +3550,7 @@
         <v>166</v>
       </c>
       <c r="B164">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C164">
         <v>0</v>
@@ -3564,7 +3564,7 @@
         <v>167</v>
       </c>
       <c r="B165">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C165">
         <v>0</v>
@@ -3578,7 +3578,7 @@
         <v>168</v>
       </c>
       <c r="B166">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C166">
         <v>0</v>
@@ -3592,7 +3592,7 @@
         <v>169</v>
       </c>
       <c r="B167">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C167">
         <v>0</v>
@@ -3623,10 +3623,10 @@
         <v>64</v>
       </c>
       <c r="C169">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="D169" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -3648,7 +3648,7 @@
         <v>173</v>
       </c>
       <c r="B171">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C171">
         <v>0</v>
@@ -3662,7 +3662,7 @@
         <v>174</v>
       </c>
       <c r="B172">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C172">
         <v>0</v>
@@ -3676,7 +3676,7 @@
         <v>175</v>
       </c>
       <c r="B173">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C173">
         <v>0</v>
@@ -3690,13 +3690,13 @@
         <v>176</v>
       </c>
       <c r="B174">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C174">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="D174" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -3704,7 +3704,7 @@
         <v>177</v>
       </c>
       <c r="B175">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C175">
         <v>0</v>
@@ -3718,7 +3718,7 @@
         <v>178</v>
       </c>
       <c r="B176">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C176">
         <v>0</v>
@@ -3732,7 +3732,7 @@
         <v>179</v>
       </c>
       <c r="B177">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C177">
         <v>0</v>
@@ -3746,7 +3746,7 @@
         <v>180</v>
       </c>
       <c r="B178">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C178">
         <v>0</v>
@@ -3760,7 +3760,7 @@
         <v>181</v>
       </c>
       <c r="B179">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C179">
         <v>0</v>
@@ -3774,7 +3774,7 @@
         <v>182</v>
       </c>
       <c r="B180">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C180">
         <v>0</v>
@@ -3788,7 +3788,7 @@
         <v>183</v>
       </c>
       <c r="B181">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C181">
         <v>0</v>
@@ -3802,7 +3802,7 @@
         <v>184</v>
       </c>
       <c r="B182">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C182">
         <v>0</v>
@@ -3816,7 +3816,7 @@
         <v>185</v>
       </c>
       <c r="B183">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C183">
         <v>0</v>
@@ -3830,7 +3830,7 @@
         <v>186</v>
       </c>
       <c r="B184">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C184">
         <v>0</v>
@@ -3844,7 +3844,7 @@
         <v>187</v>
       </c>
       <c r="B185">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C185">
         <v>0</v>
@@ -3858,7 +3858,7 @@
         <v>188</v>
       </c>
       <c r="B186">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C186">
         <v>0</v>
@@ -3872,7 +3872,7 @@
         <v>189</v>
       </c>
       <c r="B187">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C187">
         <v>0</v>
@@ -3886,7 +3886,7 @@
         <v>190</v>
       </c>
       <c r="B188">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C188">
         <v>0</v>
@@ -3900,7 +3900,7 @@
         <v>191</v>
       </c>
       <c r="B189">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C189">
         <v>0</v>
@@ -3914,7 +3914,7 @@
         <v>192</v>
       </c>
       <c r="B190">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C190">
         <v>0</v>
@@ -3928,7 +3928,7 @@
         <v>193</v>
       </c>
       <c r="B191">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C191">
         <v>0</v>
@@ -3942,7 +3942,7 @@
         <v>194</v>
       </c>
       <c r="B192">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C192">
         <v>0</v>
@@ -3956,7 +3956,7 @@
         <v>195</v>
       </c>
       <c r="B193">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C193">
         <v>0</v>
@@ -3970,7 +3970,7 @@
         <v>196</v>
       </c>
       <c r="B194">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C194">
         <v>0</v>
@@ -3984,7 +3984,7 @@
         <v>197</v>
       </c>
       <c r="B195">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C195">
         <v>0</v>
@@ -3998,7 +3998,7 @@
         <v>198</v>
       </c>
       <c r="B196">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C196">
         <v>0</v>
@@ -4012,7 +4012,7 @@
         <v>199</v>
       </c>
       <c r="B197">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C197">
         <v>0</v>
@@ -4026,7 +4026,7 @@
         <v>200</v>
       </c>
       <c r="B198">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C198">
         <v>0</v>
@@ -4040,7 +4040,7 @@
         <v>201</v>
       </c>
       <c r="B199">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C199">
         <v>0</v>
@@ -4054,7 +4054,7 @@
         <v>202</v>
       </c>
       <c r="B200">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C200">
         <v>0</v>
@@ -4068,7 +4068,7 @@
         <v>203</v>
       </c>
       <c r="B201">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C201">
         <v>0</v>
@@ -4099,7 +4099,7 @@
         <v>0</v>
       </c>
       <c r="C203">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D203" t="s">
         <v>304</v>
@@ -4113,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="C204">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D204" t="s">
         <v>304</v>
@@ -4127,7 +4127,7 @@
         <v>0</v>
       </c>
       <c r="C205">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D205" t="s">
         <v>304</v>
@@ -4141,7 +4141,7 @@
         <v>0</v>
       </c>
       <c r="C206">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D206" t="s">
         <v>304</v>
@@ -4155,7 +4155,7 @@
         <v>0</v>
       </c>
       <c r="C207">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D207" t="s">
         <v>304</v>
@@ -4183,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="C209">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D209" t="s">
         <v>304</v>
@@ -4197,7 +4197,7 @@
         <v>0</v>
       </c>
       <c r="C210">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D210" t="s">
         <v>304</v>
@@ -4211,7 +4211,7 @@
         <v>0</v>
       </c>
       <c r="C211">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D211" t="s">
         <v>304</v>
@@ -4225,7 +4225,7 @@
         <v>0</v>
       </c>
       <c r="C212">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D212" t="s">
         <v>304</v>
@@ -4239,7 +4239,7 @@
         <v>0</v>
       </c>
       <c r="C213">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D213" t="s">
         <v>304</v>
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="C214">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D214" t="s">
         <v>304</v>
@@ -4267,7 +4267,7 @@
         <v>0</v>
       </c>
       <c r="C215">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D215" t="s">
         <v>304</v>
@@ -4281,7 +4281,7 @@
         <v>0</v>
       </c>
       <c r="C216">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D216" t="s">
         <v>304</v>
@@ -4295,7 +4295,7 @@
         <v>0</v>
       </c>
       <c r="C217">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D217" t="s">
         <v>304</v>
@@ -4309,7 +4309,7 @@
         <v>0</v>
       </c>
       <c r="C218">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D218" t="s">
         <v>304</v>
@@ -4323,7 +4323,7 @@
         <v>0</v>
       </c>
       <c r="C219">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D219" t="s">
         <v>304</v>
@@ -4337,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="C220">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D220" t="s">
         <v>304</v>
@@ -4351,7 +4351,7 @@
         <v>0</v>
       </c>
       <c r="C221">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D221" t="s">
         <v>304</v>
@@ -4365,7 +4365,7 @@
         <v>0</v>
       </c>
       <c r="C222">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D222" t="s">
         <v>304</v>
@@ -4379,7 +4379,7 @@
         <v>0</v>
       </c>
       <c r="C223">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D223" t="s">
         <v>304</v>
@@ -4393,7 +4393,7 @@
         <v>0</v>
       </c>
       <c r="C224">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D224" t="s">
         <v>304</v>
@@ -4407,7 +4407,7 @@
         <v>0</v>
       </c>
       <c r="C225">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D225" t="s">
         <v>304</v>
@@ -4421,7 +4421,7 @@
         <v>0</v>
       </c>
       <c r="C226">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D226" t="s">
         <v>304</v>
@@ -4435,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="C227">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D227" t="s">
         <v>304</v>
@@ -4449,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="C228">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D228" t="s">
         <v>304</v>
@@ -4463,7 +4463,7 @@
         <v>0</v>
       </c>
       <c r="C229">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D229" t="s">
         <v>304</v>
@@ -4505,7 +4505,7 @@
         <v>0</v>
       </c>
       <c r="C232">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D232" t="s">
         <v>304</v>
@@ -4519,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="C233">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D233" t="s">
         <v>304</v>
@@ -4533,7 +4533,7 @@
         <v>0</v>
       </c>
       <c r="C234">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D234" t="s">
         <v>304</v>
@@ -4547,7 +4547,7 @@
         <v>0</v>
       </c>
       <c r="C235">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D235" t="s">
         <v>304</v>
@@ -4561,7 +4561,7 @@
         <v>0</v>
       </c>
       <c r="C236">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D236" t="s">
         <v>304</v>
@@ -4575,7 +4575,7 @@
         <v>0</v>
       </c>
       <c r="C237">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D237" t="s">
         <v>304</v>
@@ -4589,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="C238">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D238" t="s">
         <v>304</v>
@@ -4603,7 +4603,7 @@
         <v>0</v>
       </c>
       <c r="C239">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D239" t="s">
         <v>304</v>
@@ -4617,7 +4617,7 @@
         <v>0</v>
       </c>
       <c r="C240">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D240" t="s">
         <v>304</v>
@@ -4631,7 +4631,7 @@
         <v>0</v>
       </c>
       <c r="C241">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D241" t="s">
         <v>304</v>
@@ -4645,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="C242">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D242" t="s">
         <v>304</v>
@@ -4673,7 +4673,7 @@
         <v>0</v>
       </c>
       <c r="C244">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D244" t="s">
         <v>304</v>
@@ -4687,7 +4687,7 @@
         <v>0</v>
       </c>
       <c r="C245">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D245" t="s">
         <v>304</v>
@@ -4701,7 +4701,7 @@
         <v>0</v>
       </c>
       <c r="C246">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D246" t="s">
         <v>304</v>
@@ -4715,7 +4715,7 @@
         <v>0</v>
       </c>
       <c r="C247">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D247" t="s">
         <v>304</v>
@@ -4729,7 +4729,7 @@
         <v>0</v>
       </c>
       <c r="C248">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D248" t="s">
         <v>304</v>
@@ -4743,7 +4743,7 @@
         <v>0</v>
       </c>
       <c r="C249">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D249" t="s">
         <v>304</v>
@@ -4757,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="C250">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D250" t="s">
         <v>304</v>
@@ -4771,7 +4771,7 @@
         <v>0</v>
       </c>
       <c r="C251">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D251" t="s">
         <v>304</v>
@@ -4785,7 +4785,7 @@
         <v>0</v>
       </c>
       <c r="C252">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D252" t="s">
         <v>304</v>
@@ -4799,7 +4799,7 @@
         <v>0</v>
       </c>
       <c r="C253">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D253" t="s">
         <v>304</v>
@@ -4841,7 +4841,7 @@
         <v>0</v>
       </c>
       <c r="C256">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D256" t="s">
         <v>304</v>
@@ -4855,7 +4855,7 @@
         <v>0</v>
       </c>
       <c r="C257">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D257" t="s">
         <v>304</v>
@@ -4869,7 +4869,7 @@
         <v>0</v>
       </c>
       <c r="C258">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D258" t="s">
         <v>304</v>
@@ -4883,7 +4883,7 @@
         <v>0</v>
       </c>
       <c r="C259">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D259" t="s">
         <v>304</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="C260">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="D260" t="s">
         <v>304</v>
@@ -4911,7 +4911,7 @@
         <v>0</v>
       </c>
       <c r="C261">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D261" t="s">
         <v>304</v>
@@ -4925,7 +4925,7 @@
         <v>0</v>
       </c>
       <c r="C262">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D262" t="s">
         <v>304</v>
@@ -4939,7 +4939,7 @@
         <v>0</v>
       </c>
       <c r="C263">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D263" t="s">
         <v>304</v>
@@ -4953,7 +4953,7 @@
         <v>0</v>
       </c>
       <c r="C264">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D264" t="s">
         <v>304</v>
@@ -4967,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="C265">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D265" t="s">
         <v>304</v>
@@ -4981,7 +4981,7 @@
         <v>0</v>
       </c>
       <c r="C266">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D266" t="s">
         <v>304</v>
@@ -4995,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="C267">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D267" t="s">
         <v>304</v>
@@ -5009,7 +5009,7 @@
         <v>0</v>
       </c>
       <c r="C268">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D268" t="s">
         <v>304</v>
@@ -5023,7 +5023,7 @@
         <v>0</v>
       </c>
       <c r="C269">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D269" t="s">
         <v>304</v>
@@ -5037,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="C270">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D270" t="s">
         <v>304</v>
@@ -5051,7 +5051,7 @@
         <v>0</v>
       </c>
       <c r="C271">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D271" t="s">
         <v>304</v>
@@ -5065,7 +5065,7 @@
         <v>0</v>
       </c>
       <c r="C272">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D272" t="s">
         <v>304</v>
@@ -5079,7 +5079,7 @@
         <v>0</v>
       </c>
       <c r="C273">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D273" t="s">
         <v>304</v>
@@ -5093,7 +5093,7 @@
         <v>0</v>
       </c>
       <c r="C274">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D274" t="s">
         <v>304</v>
@@ -5107,7 +5107,7 @@
         <v>0</v>
       </c>
       <c r="C275">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D275" t="s">
         <v>304</v>
@@ -5121,7 +5121,7 @@
         <v>0</v>
       </c>
       <c r="C276">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D276" t="s">
         <v>304</v>
@@ -5135,7 +5135,7 @@
         <v>0</v>
       </c>
       <c r="C277">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D277" t="s">
         <v>304</v>
@@ -5149,7 +5149,7 @@
         <v>0</v>
       </c>
       <c r="C278">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D278" t="s">
         <v>304</v>
@@ -5163,7 +5163,7 @@
         <v>0</v>
       </c>
       <c r="C279">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D279" t="s">
         <v>304</v>
@@ -5177,7 +5177,7 @@
         <v>0</v>
       </c>
       <c r="C280">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D280" t="s">
         <v>304</v>
@@ -5191,7 +5191,7 @@
         <v>0</v>
       </c>
       <c r="C281">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D281" t="s">
         <v>304</v>
@@ -5205,7 +5205,7 @@
         <v>0</v>
       </c>
       <c r="C282">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D282" t="s">
         <v>304</v>
@@ -5219,7 +5219,7 @@
         <v>0</v>
       </c>
       <c r="C283">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D283" t="s">
         <v>304</v>
@@ -5233,7 +5233,7 @@
         <v>0</v>
       </c>
       <c r="C284">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D284" t="s">
         <v>304</v>
@@ -5247,7 +5247,7 @@
         <v>0</v>
       </c>
       <c r="C285">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D285" t="s">
         <v>304</v>
@@ -5261,7 +5261,7 @@
         <v>0</v>
       </c>
       <c r="C286">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D286" t="s">
         <v>304</v>
@@ -5275,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="C287">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D287" t="s">
         <v>304</v>
@@ -5289,7 +5289,7 @@
         <v>0</v>
       </c>
       <c r="C288">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D288" t="s">
         <v>304</v>
@@ -5303,7 +5303,7 @@
         <v>0</v>
       </c>
       <c r="C289">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D289" t="s">
         <v>304</v>
@@ -5317,7 +5317,7 @@
         <v>0</v>
       </c>
       <c r="C290">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D290" t="s">
         <v>304</v>
@@ -5331,7 +5331,7 @@
         <v>0</v>
       </c>
       <c r="C291">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D291" t="s">
         <v>304</v>
@@ -5345,7 +5345,7 @@
         <v>0</v>
       </c>
       <c r="C292">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D292" t="s">
         <v>304</v>
@@ -5359,7 +5359,7 @@
         <v>0</v>
       </c>
       <c r="C293">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D293" t="s">
         <v>304</v>
@@ -5373,7 +5373,7 @@
         <v>0</v>
       </c>
       <c r="C294">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D294" t="s">
         <v>304</v>
@@ -5387,7 +5387,7 @@
         <v>0</v>
       </c>
       <c r="C295">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D295" t="s">
         <v>304</v>
@@ -5401,7 +5401,7 @@
         <v>0</v>
       </c>
       <c r="C296">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D296" t="s">
         <v>304</v>
@@ -5415,7 +5415,7 @@
         <v>0</v>
       </c>
       <c r="C297">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D297" t="s">
         <v>304</v>
@@ -5429,7 +5429,7 @@
         <v>0</v>
       </c>
       <c r="C298">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D298" t="s">
         <v>304</v>
@@ -5443,7 +5443,7 @@
         <v>0</v>
       </c>
       <c r="C299">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D299" t="s">
         <v>304</v>

</xml_diff>